<commit_message>
commit "push to github"
</commit_message>
<xml_diff>
--- a/vTiger_Application/src/main/resources/Vtiger_Test_Data.xlsx
+++ b/vTiger_Application/src/main/resources/Vtiger_Test_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10994E9E-D8A7-43B7-BE93-6714BB8942DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191DC313-1EFB-461C-8E96-75D9CDFDA8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="1" r:id="rId1"/>
@@ -328,12 +328,6 @@
     <t xml:space="preserve">	ACC62396</t>
   </si>
   <si>
-    <t>CON33714</t>
-  </si>
-  <si>
-    <t>CON33720</t>
-  </si>
-  <si>
     <t>CON33722</t>
   </si>
   <si>
@@ -343,21 +337,12 @@
     <t xml:space="preserve">		ACC62312</t>
   </si>
   <si>
-    <t xml:space="preserve">	ACC62315</t>
-  </si>
-  <si>
-    <t xml:space="preserve">	 ACC62316</t>
-  </si>
-  <si>
     <t xml:space="preserve">	ACC62319</t>
   </si>
   <si>
     <t>ACC62321</t>
   </si>
   <si>
-    <t>CON33713</t>
-  </si>
-  <si>
     <t>CON33725</t>
   </si>
   <si>
@@ -365,6 +350,21 @@
   </si>
   <si>
     <t>CON337027</t>
+  </si>
+  <si>
+    <t>CON33731</t>
+  </si>
+  <si>
+    <t>CON33732</t>
+  </si>
+  <si>
+    <t>CON33733</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	ACC62317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	 ACC62318</t>
   </si>
 </sst>
 </file>
@@ -983,7 +983,7 @@
         <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -991,7 +991,7 @@
         <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -999,7 +999,7 @@
         <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1007,7 +1007,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1023,7 +1023,7 @@
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1104,7 +1104,7 @@
         <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -1112,7 +1112,7 @@
         <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -1120,7 +1120,7 @@
         <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
@@ -1128,7 +1128,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
@@ -1136,7 +1136,7 @@
         <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -1144,7 +1144,7 @@
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -1152,7 +1152,7 @@
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -1160,7 +1160,7 @@
         <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>